<commit_message>
RF04a: risco, reserva atômica no MO e SAGA FO↔MO por outbox/Kafka
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/ordens.xlsx
+++ b/frontend/runner/exemplos/ordens.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="76">
   <si>
     <t>cenario</t>
   </si>
@@ -201,7 +201,7 @@
     <t>{"cache-control":"no-store"}</t>
   </si>
   <si>
-    <t>{"/id":"${id}","/tipo":"LIMIT","/validade":"DIA","/estado":"RECEBIDA"}</t>
+    <t>{"/id":"${id}","/tipo":"LIMIT","/validade":"DIA","/estado":"RESERVADA","/motivoRejeicao":null}</t>
   </si>
   <si>
     <t>{}</t>
@@ -904,11 +904,11 @@
       <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>19</v>
+      <c r="J2">
+        <v>200</v>
+      </c>
+      <c r="K2">
+        <v>15000</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
RF05c.3b2: isola pares vivos em DELTA3 e repete guardas do par no MO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/ordens.xlsx
+++ b/frontend/runner/exemplos/ordens.xlsx
@@ -105,7 +105,7 @@
     <t>/api/v1/ordens-oco</t>
   </si>
   <si>
-    <t>{"ticker":"BETA3","lado":"VENDA","quantidade":50,"validade":"DIA","takeProfit":{"precoLimite":"21.00"},"stopLoss":{"tipo":"STOP","precoGatilho":"19.00"}}</t>
+    <t>{"ticker":"DELTA3","lado":"VENDA","quantidade":50,"validade":"DIA","takeProfit":{"precoLimite":"42.00"},"stopLoss":{"tipo":"STOP","precoGatilho":"38.00"}}</t>
   </si>
   <si>
     <t>{"grupo":"/grupoOco"}</t>
@@ -237,7 +237,7 @@
     <t>{"/ordens/0/papelOco":"TAKE_PROFIT","/ordens/1/papelOco":"STOP_LOSS"}</t>
   </si>
   <si>
-    <t>{"/grupoOco":"${grupo}","/ordens/0/tipo":"LIMIT","/ordens/1/tipo":"STOP","/ordens/1/precoGatilho":"19.00"}</t>
+    <t>{"/grupoOco":"${grupo}","/ordens/0/tipo":"LIMIT","/ordens/1/tipo":"STOP","/ordens/1/precoGatilho":"38.00"}</t>
   </si>
   <si>
     <t>{"/codigo":"GRUPO_OCO_NAO_ENCONTRADO"}</t>

</xml_diff>